<commit_message>
FINAL CODE FOR ADVENTUS IT SERVICES - FUNCTIONALITY ADDITIONS and iterations, UI additions.
</commit_message>
<xml_diff>
--- a/excel_exports/warehouse_1/Acer_Defective.xlsx
+++ b/excel_exports/warehouse_1/Acer_Defective.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-26 08:07:42</t>
+          <t>2026-04-26 22:22:25</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PS-0117</t>
+          <t>PS-1000</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>NXBHSSP00122114444</t>
+          <t>NXBHSSP001221176522</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -481,7 +481,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Area C</t>
+          <t>Area A</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -491,29 +491,29 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Defective Keys</t>
+          <t>No Display</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-04-25 23:12:00</t>
+          <t>2026-04-26 22:15:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-26 08:07:42</t>
+          <t>2026-04-26 22:22:25</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PS-0122</t>
+          <t>PS-2000</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>NXBHSSP00122117611</t>
+          <t>NXBHSSP001221176533</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -523,7 +523,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Area C</t>
+          <t>Area A</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -538,24 +538,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-04-25 23:12:00</t>
+          <t>2026-04-26 22:15:40</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-26 08:08:23</t>
+          <t>2026-04-26 22:22:25</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>PS-0100</t>
+          <t>PS-3000</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>NXBHSSP00122117666</t>
+          <t>NXBHSSP001221176544</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -565,39 +565,39 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Area C</t>
+          <t>Area A</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Minimal</t>
+          <t>Defective</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Scratches</t>
+          <t>No Display</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-04-25 23:12:00</t>
+          <t>2026-04-26 22:15:40</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-26 08:08:23</t>
+          <t>2026-04-26 22:24:39</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PS-0155</t>
+          <t>PS-3100</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>NXBHSSP00122117677</t>
+          <t>NXBHSSP001221176555</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Area C</t>
+          <t>Area B</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -622,24 +622,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-04-25 23:12:00</t>
+          <t>2026-04-26 22:15:40</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-26 08:08:23</t>
+          <t>2026-04-26 22:24:39</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PS-0000</t>
+          <t>PS-3200</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>NXBHSSP00122117777</t>
+          <t>NXBHSSP001221176566</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Rack 2 - Bay 1</t>
+          <t>Area B</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -664,7 +664,49 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-04-25 23:12:00</t>
+          <t>2026-04-26 22:15:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-26 22:24:39</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PS-3300</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>NXBHSSP001221176577</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Benj</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Area B</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Minimal</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Scratches</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-04-26 22:15:40</t>
         </is>
       </c>
     </row>

</xml_diff>